<commit_message>
build phase 4 operations depth
</commit_message>
<xml_diff>
--- a/docs/Operator-Alert-Config.xlsx
+++ b/docs/Operator-Alert-Config.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="113">
   <si>
     <t>PARAMETER</t>
   </si>
@@ -249,9 +249,6 @@
   </si>
   <si>
     <t>+2348109051477</t>
-  </si>
-  <si>
-    <t>Pending</t>
   </si>
   <si>
     <t>c6ed040b-cf74-431d-9dc3-862b90ef43a5</t>
@@ -1087,7 +1084,7 @@
         <v>60000.0</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12">
@@ -1321,21 +1318,21 @@
         <v>27000.0</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>78</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>79</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>80</v>
       </c>
       <c r="C21" s="17" t="s">
         <v>25</v>
       </c>
       <c r="D21" s="20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>27</v>
@@ -1352,19 +1349,19 @@
     </row>
     <row r="22">
       <c r="A22" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>82</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>83</v>
       </c>
       <c r="C22" s="17" t="s">
         <v>25</v>
       </c>
       <c r="D22" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="E22" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>85</v>
       </c>
       <c r="F22" s="21" t="s">
         <v>38</v>
@@ -1378,16 +1375,16 @@
     </row>
     <row r="23">
       <c r="A23" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>86</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>87</v>
       </c>
       <c r="C23" s="17" t="s">
         <v>25</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>27</v>
@@ -8206,7 +8203,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="28" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>5</v>
@@ -8215,10 +8212,10 @@
         <v>7</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E1" s="28" t="s">
         <v>90</v>
-      </c>
-      <c r="E1" s="28" t="s">
-        <v>91</v>
       </c>
       <c r="F1" s="9"/>
       <c r="G1" s="9"/>
@@ -8247,13 +8244,13 @@
         <v>38</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C2" s="29" t="s">
         <v>92</v>
       </c>
-      <c r="C2" s="29" t="s">
+      <c r="D2" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>94</v>
       </c>
       <c r="E2" s="21" t="s">
         <v>38</v>
@@ -8261,16 +8258,16 @@
     </row>
     <row r="3">
       <c r="A3" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="29" t="s">
         <v>96</v>
       </c>
-      <c r="C3" s="29" t="s">
+      <c r="D3" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>98</v>
       </c>
       <c r="E3" s="21" t="s">
         <v>38</v>
@@ -8281,13 +8278,13 @@
         <v>17</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C4" s="29" t="s">
         <v>99</v>
       </c>
-      <c r="C4" s="29" t="s">
+      <c r="D4" s="2" t="s">
         <v>100</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>101</v>
       </c>
       <c r="E4" s="21" t="s">
         <v>38</v>
@@ -12295,7 +12292,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="28" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>5</v>
@@ -12304,7 +12301,7 @@
         <v>7</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E1" s="9"/>
       <c r="F1" s="9"/>
@@ -12334,13 +12331,13 @@
         <v>38</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C2" s="30" t="s">
         <v>102</v>
       </c>
-      <c r="C2" s="30" t="s">
+      <c r="D2" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="3">
@@ -15357,19 +15354,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>107</v>
       </c>
       <c r="F1" s="9"/>
       <c r="G1" s="9"/>
@@ -15398,7 +15395,7 @@
         <v>37</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C2" s="2">
         <v>6.44487546164212</v>
@@ -15412,10 +15409,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>110</v>
       </c>
       <c r="C3" s="2">
         <v>6.56214734154072</v>
@@ -15429,10 +15426,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C4" s="2">
         <v>6.43226684371674</v>
@@ -15449,7 +15446,7 @@
         <v>16</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C5" s="2">
         <v>6.63418881933445</v>
@@ -15466,7 +15463,7 @@
         <v>27</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C6" s="2">
         <v>6.56694136811928</v>

</xml_diff>